<commit_message>
Logistic Regression structure uploaded
</commit_message>
<xml_diff>
--- a/ML/Regression/Logistic_Regression/Logistic Regression.xlsx
+++ b/ML/Regression/Logistic_Regression/Logistic Regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Assignment\Chirag\Uploads\Assignment\ML\Regression\Logistic_Regression\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DBF6AF0-26A5-45AB-9607-7D81BB52AA9D}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="41" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09763852-C44B-4F12-8471-CBF95B07C0D0}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="41" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1080" yWindow="1080" windowWidth="15375" windowHeight="7785" xr2:uid="{0380573A-65B2-4152-9E5A-5C53E7583A18}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{0380573A-65B2-4152-9E5A-5C53E7583A18}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -151,7 +151,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -167,6 +167,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -585,11 +593,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
@@ -633,15 +638,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -967,136 +981,136 @@
     <col min="6" max="6" width="24.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="33" t="s">
+    <row r="1" spans="2:8" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36"/>
-      <c r="H1" s="34"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
+      <c r="G1" s="37"/>
+      <c r="H1" s="38"/>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
+      <c r="C3" s="35"/>
+      <c r="D3" s="35"/>
+      <c r="E3" s="35"/>
+      <c r="F3" s="35"/>
     </row>
     <row r="4" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="35" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
+      <c r="E4" s="35"/>
+      <c r="F4" s="35"/>
     </row>
     <row r="5" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="6" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="7" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="7" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="13" t="s">
+      <c r="C7" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="D7" s="13" t="s">
+      <c r="D7" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="E7" s="14" t="s">
+      <c r="E7" s="13" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B8" s="9">
+      <c r="B8" s="8">
         <v>1</v>
       </c>
-      <c r="C8" s="10">
+      <c r="C8" s="9">
         <v>1.4</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="E8" s="11">
+      <c r="E8" s="10">
         <v>1</v>
       </c>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B9" s="3">
+      <c r="B9" s="2">
         <v>2</v>
       </c>
-      <c r="C9" s="2">
+      <c r="C9" s="1">
         <v>1.5</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E9" s="4">
+      <c r="E9" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B10" s="3">
+      <c r="B10" s="2">
         <v>3</v>
       </c>
-      <c r="C10" s="2">
+      <c r="C10" s="1">
         <v>1.3</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E10" s="4">
+      <c r="E10" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B11" s="3">
+      <c r="B11" s="2">
         <v>4</v>
       </c>
-      <c r="C11" s="2">
+      <c r="C11" s="1">
         <v>4.5</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E11" s="4">
+      <c r="E11" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="5">
+      <c r="B12" s="4">
         <v>5</v>
       </c>
-      <c r="C12" s="6">
+      <c r="C12" s="5">
         <v>5.0999999999999996</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="D12" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E12" s="7">
+      <c r="E12" s="6">
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C14" s="31" t="s">
+      <c r="C14" s="30" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="15" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C15" s="32" t="s">
+      <c r="C15" s="31" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1107,7 +1121,7 @@
       <c r="C16" s="34"/>
     </row>
     <row r="17" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C17" s="35" t="s">
+      <c r="C17" s="32" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1121,100 +1135,100 @@
       <c r="C19" t="s">
         <v>14</v>
       </c>
-      <c r="F19" s="15"/>
-      <c r="G19" s="15"/>
-    </row>
-    <row r="20" spans="1:7" s="23" customFormat="1" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C20" s="24" t="s">
+      <c r="F19" s="14"/>
+      <c r="G19" s="14"/>
+    </row>
+    <row r="20" spans="1:7" s="22" customFormat="1" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C20" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="D20" s="26" t="s">
+      <c r="D20" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="E20" s="27" t="s">
+      <c r="E20" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="F20" s="25" t="s">
+      <c r="F20" s="24" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C21" s="20">
+      <c r="C21" s="19">
         <v>1.4</v>
       </c>
-      <c r="D21" s="16">
+      <c r="D21" s="15">
         <f xml:space="preserve"> -3 * C21 + 7</f>
         <v>2.8000000000000007</v>
       </c>
-      <c r="E21" s="28">
+      <c r="E21" s="27">
         <f xml:space="preserve"> 1 / (1 + 2.71 ^(-D21))</f>
         <v>0.94221238206586821</v>
       </c>
-      <c r="F21" s="28" t="s">
+      <c r="F21" s="27" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C22" s="21">
+      <c r="C22" s="20">
         <v>1.5</v>
       </c>
-      <c r="D22" s="17">
+      <c r="D22" s="16">
         <f t="shared" ref="D22:D25" si="0" xml:space="preserve"> -3 * C22 + 7</f>
         <v>2.5</v>
       </c>
-      <c r="E22" s="28">
+      <c r="E22" s="27">
         <f t="shared" ref="E22:E25" si="1" xml:space="preserve"> 1 / (1 + 2.71 ^(-D22))</f>
         <v>0.92360530658936724</v>
       </c>
-      <c r="F22" s="29" t="s">
+      <c r="F22" s="28" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C23" s="21">
+      <c r="C23" s="20">
         <v>1.3</v>
       </c>
-      <c r="D23" s="17">
+      <c r="D23" s="16">
         <f t="shared" si="0"/>
         <v>3.0999999999999996</v>
       </c>
-      <c r="E23" s="28">
+      <c r="E23" s="27">
         <f t="shared" si="1"/>
         <v>0.95650087031673725</v>
       </c>
-      <c r="F23" s="29" t="s">
+      <c r="F23" s="28" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C24" s="21">
+      <c r="C24" s="20">
         <v>4.5</v>
       </c>
-      <c r="D24" s="17">
+      <c r="D24" s="16">
         <f t="shared" si="0"/>
         <v>-6.5</v>
       </c>
-      <c r="E24" s="28">
+      <c r="E24" s="27">
         <f xml:space="preserve"> 1 / (1 + 2.71 ^(-D24))</f>
         <v>1.5312077008417307E-3</v>
       </c>
-      <c r="F24" s="29" t="s">
+      <c r="F24" s="28" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C25" s="22">
+      <c r="C25" s="21">
         <v>5.0999999999999996</v>
       </c>
-      <c r="D25" s="18">
+      <c r="D25" s="17">
         <f t="shared" si="0"/>
         <v>-8.2999999999999989</v>
       </c>
-      <c r="E25" s="19">
+      <c r="E25" s="18">
         <f t="shared" si="1"/>
         <v>2.5482627274268574E-4</v>
       </c>
-      <c r="F25" s="30" t="s">
+      <c r="F25" s="29" t="s">
         <v>21</v>
       </c>
     </row>

</xml_diff>